<commit_message>
Add reconciliation layer: dbt models, ebook sections, Excel tab
- int_payment_reconciliation + int_payout_reconciliation (Silver intermediate)
- mart_reconciliation (Gold, grain: business × corridor × month)
- assert_gold_remittance_volume_matches_bronze singular test
- Ebook: sections 4.7 Reconciliation Controls, 5.5 mart_reconciliation, 7.3 Reconciliation KPIs
- Excel: new Reconciliation & Settlement Controls tab
- scripts/step2_excel.py: BASE path fixed to relative; reconciliation tab added
- Replaced generic_tests.yml with model-level YAML docs
</commit_message>
<xml_diff>
--- a/excel/AfriMoney_Dashboard.xlsx
+++ b/excel/AfriMoney_Dashboard.xlsx
@@ -13,10 +13,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer 360" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Profitability" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk &amp; Compliance" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AfriMoney Lending" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet &amp; Card" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Model" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AfriMoney Lending" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet &amp; Card" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Model" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -230,6 +231,12 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
+      <color rgb="00FF6B6B"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
       <color rgb="0000C97A"/>
       <sz val="16"/>
     </font>
@@ -237,12 +244,6 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00F5A623"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FF6B6B"/>
       <sz val="16"/>
     </font>
     <font>
@@ -403,7 +404,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -547,16 +548,13 @@
     <xf numFmtId="0" fontId="32" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -568,10 +566,19 @@
     <xf numFmtId="0" fontId="35" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="31" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="36" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -584,10 +591,10 @@
     <xf numFmtId="0" fontId="37" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="38" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="38" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2323,7 +2330,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Snowflake · dbt · Snowpark ML  |  Reporting Period: 2025–2026  |  Generated: 2026-06-30</t>
+          <t>Snowflake · dbt · Snowpark ML  |  Reporting Period: 2025–2026  |  Generated: 2026-08-19</t>
         </is>
       </c>
     </row>
@@ -2675,6 +2682,773 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="000D2137"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:K26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="B1" s="22" t="inlineStr">
+        <is>
+          <t>AfriMoney — Snowflake Data Model (Bronze→Silver→Gold)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1"/>
+    <row r="4" ht="32" customHeight="1">
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Schema</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Table Name</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Row Count</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>Key Column</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>Key Fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>BRONZE</t>
+        </is>
+      </c>
+      <c r="C5" s="66" t="inlineStr">
+        <is>
+          <t>dim_customer</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>500,000</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>SCD2</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>customer_sk</t>
+        </is>
+      </c>
+      <c r="G5" s="36" t="inlineStr">
+        <is>
+          <t>customer_id, kyc_level, risk_band, status</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>BRONZE</t>
+        </is>
+      </c>
+      <c r="C6" s="67" t="inlineStr">
+        <is>
+          <t>dim_recipient</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>1,000,000</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>Dimension</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>recipient_id</t>
+        </is>
+      </c>
+      <c r="G6" s="37" t="inlineStr">
+        <is>
+          <t>name_hash, country, payout_method</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>BRONZE</t>
+        </is>
+      </c>
+      <c r="C7" s="66" t="inlineStr">
+        <is>
+          <t>fact_remittance_transfer</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>5,000,000</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>Fact</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>transfer_id</t>
+        </is>
+      </c>
+      <c r="G7" s="36" t="inlineStr">
+        <is>
+          <t>send_amt_zar, corridor, channel, status</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>BRONZE</t>
+        </is>
+      </c>
+      <c r="C8" s="67" t="inlineStr">
+        <is>
+          <t>fact_wallet_ledger</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>~10,000,000</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>Fact (double-entry)</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>ledger_id</t>
+        </is>
+      </c>
+      <c r="G8" s="37" t="inlineStr">
+        <is>
+          <t>customer_id, direction, amount, type</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>BRONZE</t>
+        </is>
+      </c>
+      <c r="C9" s="66" t="inlineStr">
+        <is>
+          <t>fact_card_transaction</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>~3,000,000</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>Fact</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>txn_id</t>
+        </is>
+      </c>
+      <c r="G9" s="36" t="inlineStr">
+        <is>
+          <t>amount, status, merchant, fraud_flag</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>BRONZE</t>
+        </is>
+      </c>
+      <c r="C10" s="67" t="inlineStr">
+        <is>
+          <t>fact_loan_application</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>200,000</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>Fact</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>loan_id</t>
+        </is>
+      </c>
+      <c r="G10" s="37" t="inlineStr">
+        <is>
+          <t>principal, decision, dpd, pd_score</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>BRONZE</t>
+        </is>
+      </c>
+      <c r="C11" s="66" t="inlineStr">
+        <is>
+          <t>fact_fx_rate</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>~95,000</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>Fact</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>rate_id</t>
+        </is>
+      </c>
+      <c r="G11" s="36" t="inlineStr">
+        <is>
+          <t>corridor, interbank, applied, spread_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>BRONZE</t>
+        </is>
+      </c>
+      <c r="C12" s="67" t="inlineStr">
+        <is>
+          <t>fact_insurance_policy</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>40,000</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>Fact</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>policy_id</t>
+        </is>
+      </c>
+      <c r="G12" s="37" t="inlineStr">
+        <is>
+          <t>product, premium, status</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>BRONZE</t>
+        </is>
+      </c>
+      <c r="C13" s="66" t="inlineStr">
+        <is>
+          <t>fact_usd_savings</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>Fact</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>account_id</t>
+        </is>
+      </c>
+      <c r="G13" s="36" t="inlineStr">
+        <is>
+          <t>balance_zar, usdc_balance, status</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="B14" s="25" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="C14" s="67" t="inlineStr">
+        <is>
+          <t>stg_transfers</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>view</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>dbt view</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="37" t="inlineStr">
+        <is>
+          <t>Cleaned transfers + derived fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="C15" s="66" t="inlineStr">
+        <is>
+          <t>int_transfer_profitability</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>~5M</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>dbt table</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" s="36" t="inlineStr">
+        <is>
+          <t>Transfers + FX join + margin tiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="B16" s="25" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="C16" s="67" t="inlineStr">
+        <is>
+          <t>int_customer_transfer_stats</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>~500K</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>dbt table</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="37" t="inlineStr">
+        <is>
+          <t>Aggregated customer behaviour</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="C17" s="66" t="inlineStr">
+        <is>
+          <t>int_payment_reconciliation</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>~5M</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>dbt table</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>transfer_id</t>
+        </is>
+      </c>
+      <c r="G17" s="36" t="inlineStr">
+        <is>
+          <t>Collected vs committed, per transfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="B18" s="25" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="C18" s="67" t="inlineStr">
+        <is>
+          <t>int_payout_reconciliation</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>~4.4M</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>dbt table</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>transfer_id</t>
+        </is>
+      </c>
+      <c r="G18" s="37" t="inlineStr">
+        <is>
+          <t>Disbursed vs committed, per transfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="C19" s="66" t="inlineStr">
+        <is>
+          <t>mart_remittance</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>~50K</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>dbt table</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" s="36" t="inlineStr">
+        <is>
+          <t>Monthly corridor KPIs + revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="C20" s="67" t="inlineStr">
+        <is>
+          <t>mart_customer_360</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>~500K</t>
+        </is>
+      </c>
+      <c r="E20" s="19" t="inlineStr">
+        <is>
+          <t>dbt table</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G20" s="37" t="inlineStr">
+        <is>
+          <t>One row per customer + LTV/engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="B21" s="23" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="C21" s="66" t="inlineStr">
+        <is>
+          <t>mart_fx_profitability</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>~200</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>dbt table</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="36" t="inlineStr">
+        <is>
+          <t>Corridor FX margin by month</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="C22" s="67" t="inlineStr">
+        <is>
+          <t>mart_risk_compliance</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>~12</t>
+        </is>
+      </c>
+      <c r="E22" s="19" t="inlineStr">
+        <is>
+          <t>dbt table</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="37" t="inlineStr">
+        <is>
+          <t>Monthly risk RAG status KPIs</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="C23" s="66" t="inlineStr">
+        <is>
+          <t>mart_loans_mukuru</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>~1K</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>dbt table</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G23" s="36" t="inlineStr">
+        <is>
+          <t>Loan origination + ECL + repayment</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="B24" s="24" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="C24" s="67" t="inlineStr">
+        <is>
+          <t>mart_reconciliation</t>
+        </is>
+      </c>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>~200</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="inlineStr">
+        <is>
+          <t>dbt table</t>
+        </is>
+      </c>
+      <c r="F24" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" s="37" t="inlineStr">
+        <is>
+          <t>Monthly collection/settlement completeness</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="B25" s="68" t="inlineStr">
+        <is>
+          <t>ML_DB</t>
+        </is>
+      </c>
+      <c r="C25" s="66" t="inlineStr">
+        <is>
+          <t>FRAUD_FEATURES</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>~200K</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>Feature table</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="36" t="inlineStr">
+        <is>
+          <t>15 fraud features refreshed daily</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="69" t="inlineStr">
+        <is>
+          <t>ML_DB</t>
+        </is>
+      </c>
+      <c r="C26" s="67" t="inlineStr">
+        <is>
+          <t>CHURN_FEATURES</t>
+        </is>
+      </c>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>~500K</t>
+        </is>
+      </c>
+      <c r="E26" s="19" t="inlineStr">
+        <is>
+          <t>Feature table</t>
+        </is>
+      </c>
+      <c r="F26" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G26" s="37" t="inlineStr">
+        <is>
+          <t>21 churn features refreshed weekly</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:K2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="0000C97A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -2687,7 +3461,7 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="68" t="inlineStr">
+      <c r="B2" s="70" t="inlineStr">
         <is>
           <t>AfriMoney Intelligence Platform</t>
         </is>
@@ -2695,174 +3469,174 @@
     </row>
     <row r="3"/>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="69" t="inlineStr">
+      <c r="B5" s="71" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="C5" s="70" t="inlineStr">
+      <c r="C5" s="72" t="inlineStr">
         <is>
           <t>AfriMoney Intelligence Platform — African Remittance Analytics</t>
         </is>
       </c>
-      <c r="D5" s="71" t="n"/>
-      <c r="E5" s="71" t="n"/>
-      <c r="F5" s="71" t="n"/>
-      <c r="G5" s="71" t="n"/>
-      <c r="H5" s="72" t="n"/>
+      <c r="D5" s="73" t="n"/>
+      <c r="E5" s="73" t="n"/>
+      <c r="F5" s="73" t="n"/>
+      <c r="G5" s="73" t="n"/>
+      <c r="H5" s="74" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="69" t="inlineStr">
+      <c r="B6" s="71" t="inlineStr">
         <is>
           <t>Author</t>
         </is>
       </c>
-      <c r="C6" s="70" t="inlineStr">
+      <c r="C6" s="72" t="inlineStr">
         <is>
           <t>Anthony Apollis</t>
         </is>
       </c>
-      <c r="D6" s="71" t="n"/>
-      <c r="E6" s="71" t="n"/>
-      <c r="F6" s="71" t="n"/>
-      <c r="G6" s="71" t="n"/>
-      <c r="H6" s="72" t="n"/>
+      <c r="D6" s="73" t="n"/>
+      <c r="E6" s="73" t="n"/>
+      <c r="F6" s="73" t="n"/>
+      <c r="G6" s="73" t="n"/>
+      <c r="H6" s="74" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="69" t="inlineStr">
+      <c r="B7" s="71" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C7" s="70" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="D7" s="71" t="n"/>
-      <c r="E7" s="71" t="n"/>
-      <c r="F7" s="71" t="n"/>
-      <c r="G7" s="71" t="n"/>
-      <c r="H7" s="72" t="n"/>
+      <c r="C7" s="72" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="D7" s="73" t="n"/>
+      <c r="E7" s="73" t="n"/>
+      <c r="F7" s="73" t="n"/>
+      <c r="G7" s="73" t="n"/>
+      <c r="H7" s="74" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="69" t="inlineStr">
+      <c r="B8" s="71" t="inlineStr">
         <is>
           <t>Tech Stack</t>
         </is>
       </c>
-      <c r="C8" s="70" t="inlineStr">
+      <c r="C8" s="72" t="inlineStr">
         <is>
           <t>Snowflake · dbt · Snowpark ML · Python · Power BI</t>
         </is>
       </c>
-      <c r="D8" s="71" t="n"/>
-      <c r="E8" s="71" t="n"/>
-      <c r="F8" s="71" t="n"/>
-      <c r="G8" s="71" t="n"/>
-      <c r="H8" s="72" t="n"/>
+      <c r="D8" s="73" t="n"/>
+      <c r="E8" s="73" t="n"/>
+      <c r="F8" s="73" t="n"/>
+      <c r="G8" s="73" t="n"/>
+      <c r="H8" s="74" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="69" t="inlineStr">
+      <c r="B9" s="71" t="inlineStr">
         <is>
           <t>Architecture</t>
         </is>
       </c>
-      <c r="C9" s="70" t="inlineStr">
+      <c r="C9" s="72" t="inlineStr">
         <is>
           <t>Bronze → Silver → Gold (Medallion)</t>
         </is>
       </c>
-      <c r="D9" s="71" t="n"/>
-      <c r="E9" s="71" t="n"/>
-      <c r="F9" s="71" t="n"/>
-      <c r="G9" s="71" t="n"/>
-      <c r="H9" s="72" t="n"/>
+      <c r="D9" s="73" t="n"/>
+      <c r="E9" s="73" t="n"/>
+      <c r="F9" s="73" t="n"/>
+      <c r="G9" s="73" t="n"/>
+      <c r="H9" s="74" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="69" t="inlineStr">
+      <c r="B10" s="71" t="inlineStr">
         <is>
           <t>Data Volume</t>
         </is>
       </c>
-      <c r="C10" s="70" t="inlineStr">
+      <c r="C10" s="72" t="inlineStr">
         <is>
           <t>30M+ rows across 9 Bronze + Silver + Gold layers</t>
         </is>
       </c>
-      <c r="D10" s="71" t="n"/>
-      <c r="E10" s="71" t="n"/>
-      <c r="F10" s="71" t="n"/>
-      <c r="G10" s="71" t="n"/>
-      <c r="H10" s="72" t="n"/>
+      <c r="D10" s="73" t="n"/>
+      <c r="E10" s="73" t="n"/>
+      <c r="F10" s="73" t="n"/>
+      <c r="G10" s="73" t="n"/>
+      <c r="H10" s="74" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="69" t="inlineStr">
+      <c r="B11" s="71" t="inlineStr">
         <is>
           <t>ML Models</t>
         </is>
       </c>
-      <c r="C11" s="70" t="inlineStr">
+      <c r="C11" s="72" t="inlineStr">
         <is>
           <t>Fraud Detection (AUC 0.9582) · Churn (0.9905) · Credit PD (0.9475)</t>
         </is>
       </c>
-      <c r="D11" s="71" t="n"/>
-      <c r="E11" s="71" t="n"/>
-      <c r="F11" s="71" t="n"/>
-      <c r="G11" s="71" t="n"/>
-      <c r="H11" s="72" t="n"/>
+      <c r="D11" s="73" t="n"/>
+      <c r="E11" s="73" t="n"/>
+      <c r="F11" s="73" t="n"/>
+      <c r="G11" s="73" t="n"/>
+      <c r="H11" s="74" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="69" t="inlineStr">
+      <c r="B12" s="71" t="inlineStr">
         <is>
           <t>dbt Models</t>
         </is>
       </c>
-      <c r="C12" s="70" t="inlineStr">
-        <is>
-          <t>14 models · 28 tests passing</t>
-        </is>
-      </c>
-      <c r="D12" s="71" t="n"/>
-      <c r="E12" s="71" t="n"/>
-      <c r="F12" s="71" t="n"/>
-      <c r="G12" s="71" t="n"/>
-      <c r="H12" s="72" t="n"/>
+      <c r="C12" s="72" t="inlineStr">
+        <is>
+          <t>13 models · 41 tests passing (incl. payment &amp; settlement reconciliation)</t>
+        </is>
+      </c>
+      <c r="D12" s="73" t="n"/>
+      <c r="E12" s="73" t="n"/>
+      <c r="F12" s="73" t="n"/>
+      <c r="G12" s="73" t="n"/>
+      <c r="H12" s="74" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="69" t="inlineStr">
+      <c r="B13" s="71" t="inlineStr">
         <is>
           <t>Corridors</t>
         </is>
       </c>
-      <c r="C13" s="70" t="inlineStr">
+      <c r="C13" s="72" t="inlineStr">
         <is>
           <t>17 active SA-Africa remittance corridors</t>
         </is>
       </c>
-      <c r="D13" s="71" t="n"/>
-      <c r="E13" s="71" t="n"/>
-      <c r="F13" s="71" t="n"/>
-      <c r="G13" s="71" t="n"/>
-      <c r="H13" s="72" t="n"/>
+      <c r="D13" s="73" t="n"/>
+      <c r="E13" s="73" t="n"/>
+      <c r="F13" s="73" t="n"/>
+      <c r="G13" s="73" t="n"/>
+      <c r="H13" s="74" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="69" t="inlineStr">
+      <c r="B14" s="71" t="inlineStr">
         <is>
           <t>Disclaimer</t>
         </is>
       </c>
-      <c r="C14" s="70" t="inlineStr">
+      <c r="C14" s="72" t="inlineStr">
         <is>
           <t>Synthetic data only. No real customer data used.</t>
         </is>
       </c>
-      <c r="D14" s="71" t="n"/>
-      <c r="E14" s="71" t="n"/>
-      <c r="F14" s="71" t="n"/>
-      <c r="G14" s="71" t="n"/>
-      <c r="H14" s="72" t="n"/>
+      <c r="D14" s="73" t="n"/>
+      <c r="E14" s="73" t="n"/>
+      <c r="F14" s="73" t="n"/>
+      <c r="G14" s="73" t="n"/>
+      <c r="H14" s="74" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -5156,6 +5930,421 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FF6B6B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:K22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="B1" s="22" t="inlineStr">
+        <is>
+          <t>Reconciliation &amp; Settlement Controls — Collection vs Disbursement</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1"/>
+    <row r="3" ht="16" customHeight="1">
+      <c r="B3" s="52" t="inlineStr">
+        <is>
+          <t>mart_reconciliation (dbt Gold) — reconciles committed transfer amounts against FACT_PAYMENT (collection) and FACT_PAYOUT (settlement). Split by business unit so an over-collecting corridor can't hide an under-collecting one behind a blended average.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="14" customHeight="1">
+      <c r="B4" s="53" t="inlineStr">
+        <is>
+          <t>Collection — MKR</t>
+        </is>
+      </c>
+      <c r="D4" s="53" t="inlineStr">
+        <is>
+          <t>Collection — MMY</t>
+        </is>
+      </c>
+      <c r="F4" s="54" t="inlineStr">
+        <is>
+          <t>Settlement — MKR</t>
+        </is>
+      </c>
+      <c r="H4" s="55" t="inlineStr">
+        <is>
+          <t>Settlement — MMY</t>
+        </is>
+      </c>
+      <c r="J4" s="53" t="inlineStr">
+        <is>
+          <t>Total Recon. Breaks</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="B5" s="56" t="inlineStr">
+        <is>
+          <t>102.0%</t>
+        </is>
+      </c>
+      <c r="D5" s="56" t="inlineStr">
+        <is>
+          <t>96.5%</t>
+        </is>
+      </c>
+      <c r="F5" s="57" t="inlineStr">
+        <is>
+          <t>99.3%</t>
+        </is>
+      </c>
+      <c r="H5" s="58" t="inlineStr">
+        <is>
+          <t>96.1%</t>
+        </is>
+      </c>
+      <c r="J5" s="56" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Completed Xfers</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>Expected Collection R</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>Actual Collection R</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>Collection %</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>Committed R</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>Disbursed R</t>
+        </is>
+      </c>
+      <c r="I7" s="15" t="inlineStr">
+        <is>
+          <t>Settlement %</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>MKR</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>R 544,184.28</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>R 555,149.99</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>102.0%</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>R 530,911.43</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>R 527,190.16</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>99.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>MMY</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>R 286,639.41</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>R 276,467.48</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="inlineStr">
+        <is>
+          <t>96.5%</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>R 279,648.23</t>
+        </is>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>R 268,740.38</t>
+        </is>
+      </c>
+      <c r="I9" s="19" t="inlineStr">
+        <is>
+          <t>96.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="59" t="inlineStr">
+        <is>
+          <t>Break Types Detected (validation run)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Break Type</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="B13" s="60" t="inlineStr">
+        <is>
+          <t>MISSING_PAYMENT</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>int_payment_reconciliation</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="B14" s="61" t="inlineStr">
+        <is>
+          <t>DUPLICATE_SUCCESSFUL_PAYMENT</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>int_payment_reconciliation</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="B15" s="60" t="inlineStr">
+        <is>
+          <t>AMOUNT_MISMATCH</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>int_payment_reconciliation</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="B16" s="61" t="inlineStr">
+        <is>
+          <t>MISSING_SETTLEMENT</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>int_payout_reconciliation</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="B18" s="59" t="inlineStr">
+        <is>
+          <t>Target / Alert Thresholds</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>Alert</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="B20" s="36" t="inlineStr">
+        <is>
+          <t>Collection Completeness</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>99.5–100.5%</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>&lt;98% or &gt;102%</t>
+        </is>
+      </c>
+      <c r="E20" s="36" t="inlineStr">
+        <is>
+          <t>Finance / Treasury Ops</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="B21" s="37" t="inlineStr">
+        <is>
+          <t>Settlement Completeness</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="inlineStr">
+        <is>
+          <t>99.5–100.5%</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>&lt;98% or &gt;102%</t>
+        </is>
+      </c>
+      <c r="E21" s="37" t="inlineStr">
+        <is>
+          <t>Finance / Treasury Ops</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="36" t="inlineStr">
+        <is>
+          <t>Reconciliation Breaks</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>Any break, 2+ days running</t>
+        </is>
+      </c>
+      <c r="E22" s="36" t="inlineStr">
+        <is>
+          <t>Finance / Treasury Ops</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B1:J2"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="B4:C4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="000D2137"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -5182,32 +6371,32 @@
       </c>
     </row>
     <row r="4" ht="14" customHeight="1">
-      <c r="C4" s="53" t="inlineStr">
+      <c r="C4" s="54" t="inlineStr">
         <is>
           <t>Total Applications</t>
         </is>
       </c>
-      <c r="E4" s="54" t="inlineStr">
+      <c r="E4" s="55" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="G4" s="55" t="inlineStr">
+      <c r="G4" s="53" t="inlineStr">
         <is>
           <t>Default Rate</t>
         </is>
       </c>
-      <c r="I4" s="56" t="inlineStr">
+      <c r="I4" s="62" t="inlineStr">
         <is>
           <t>Avg Loan Size</t>
         </is>
       </c>
-      <c r="K4" s="54" t="inlineStr">
+      <c r="K4" s="55" t="inlineStr">
         <is>
           <t>IFRS 9 ECL Rate</t>
         </is>
       </c>
-      <c r="M4" s="53" t="inlineStr">
+      <c r="M4" s="54" t="inlineStr">
         <is>
           <t>AUC Credit Model</t>
         </is>
@@ -5224,12 +6413,12 @@
           <t>65%</t>
         </is>
       </c>
-      <c r="G5" s="59" t="inlineStr">
+      <c r="G5" s="56" t="inlineStr">
         <is>
           <t>11.2%</t>
         </is>
       </c>
-      <c r="I5" s="60" t="inlineStr">
+      <c r="I5" s="63" t="inlineStr">
         <is>
           <t>R 3,890</t>
         </is>
@@ -5456,7 +6645,7 @@
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="B15" s="61" t="inlineStr">
+      <c r="B15" s="59" t="inlineStr">
         <is>
           <t>Business Split — Lending Products</t>
         </is>
@@ -5579,7 +6768,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0000C97A"/>
@@ -5593,7 +6782,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="B1" s="62" t="inlineStr">
+      <c r="B1" s="64" t="inlineStr">
         <is>
           <t>Wallet &amp; Card Product Analytics</t>
         </is>
@@ -5601,37 +6790,37 @@
     </row>
     <row r="2" ht="22" customHeight="1"/>
     <row r="4" ht="32" customHeight="1">
-      <c r="B4" s="63" t="inlineStr">
+      <c r="B4" s="65" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C4" s="63" t="inlineStr">
+      <c r="C4" s="65" t="inlineStr">
         <is>
           <t>Wallet Active</t>
         </is>
       </c>
-      <c r="D4" s="63" t="inlineStr">
+      <c r="D4" s="65" t="inlineStr">
         <is>
           <t>Cash In R M</t>
         </is>
       </c>
-      <c r="E4" s="63" t="inlineStr">
+      <c r="E4" s="65" t="inlineStr">
         <is>
           <t>Cash Out R M</t>
         </is>
       </c>
-      <c r="F4" s="63" t="inlineStr">
+      <c r="F4" s="65" t="inlineStr">
         <is>
           <t>Card Txns</t>
         </is>
       </c>
-      <c r="G4" s="63" t="inlineStr">
+      <c r="G4" s="65" t="inlineStr">
         <is>
           <t>Card Spend R M</t>
         </is>
       </c>
-      <c r="H4" s="63" t="inlineStr">
+      <c r="H4" s="65" t="inlineStr">
         <is>
           <t>Card Approval %</t>
         </is>
@@ -5793,675 +6982,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="000D2137"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="B1:K23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="B1" s="22" t="inlineStr">
-        <is>
-          <t>AfriMoney — Snowflake Data Model (Bronze→Silver→Gold)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1"/>
-    <row r="4" ht="32" customHeight="1">
-      <c r="B4" s="15" t="inlineStr">
-        <is>
-          <t>Schema</t>
-        </is>
-      </c>
-      <c r="C4" s="15" t="inlineStr">
-        <is>
-          <t>Table Name</t>
-        </is>
-      </c>
-      <c r="D4" s="15" t="inlineStr">
-        <is>
-          <t>Row Count</t>
-        </is>
-      </c>
-      <c r="E4" s="15" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="F4" s="15" t="inlineStr">
-        <is>
-          <t>Key Column</t>
-        </is>
-      </c>
-      <c r="G4" s="15" t="inlineStr">
-        <is>
-          <t>Key Fields</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>BRONZE</t>
-        </is>
-      </c>
-      <c r="C5" s="64" t="inlineStr">
-        <is>
-          <t>dim_customer</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
-        <is>
-          <t>500,000</t>
-        </is>
-      </c>
-      <c r="E5" s="16" t="inlineStr">
-        <is>
-          <t>SCD2</t>
-        </is>
-      </c>
-      <c r="F5" s="16" t="inlineStr">
-        <is>
-          <t>customer_sk</t>
-        </is>
-      </c>
-      <c r="G5" s="36" t="inlineStr">
-        <is>
-          <t>customer_id, kyc_level, risk_band, status</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>BRONZE</t>
-        </is>
-      </c>
-      <c r="C6" s="65" t="inlineStr">
-        <is>
-          <t>dim_recipient</t>
-        </is>
-      </c>
-      <c r="D6" s="19" t="inlineStr">
-        <is>
-          <t>1,000,000</t>
-        </is>
-      </c>
-      <c r="E6" s="19" t="inlineStr">
-        <is>
-          <t>Dimension</t>
-        </is>
-      </c>
-      <c r="F6" s="19" t="inlineStr">
-        <is>
-          <t>recipient_id</t>
-        </is>
-      </c>
-      <c r="G6" s="37" t="inlineStr">
-        <is>
-          <t>name_hash, country, payout_method</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>BRONZE</t>
-        </is>
-      </c>
-      <c r="C7" s="64" t="inlineStr">
-        <is>
-          <t>fact_remittance_transfer</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
-        <is>
-          <t>5,000,000</t>
-        </is>
-      </c>
-      <c r="E7" s="16" t="inlineStr">
-        <is>
-          <t>Fact</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>transfer_id</t>
-        </is>
-      </c>
-      <c r="G7" s="36" t="inlineStr">
-        <is>
-          <t>send_amt_zar, corridor, channel, status</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="B8" s="21" t="inlineStr">
-        <is>
-          <t>BRONZE</t>
-        </is>
-      </c>
-      <c r="C8" s="65" t="inlineStr">
-        <is>
-          <t>fact_wallet_ledger</t>
-        </is>
-      </c>
-      <c r="D8" s="19" t="inlineStr">
-        <is>
-          <t>~10,000,000</t>
-        </is>
-      </c>
-      <c r="E8" s="19" t="inlineStr">
-        <is>
-          <t>Fact (double-entry)</t>
-        </is>
-      </c>
-      <c r="F8" s="19" t="inlineStr">
-        <is>
-          <t>ledger_id</t>
-        </is>
-      </c>
-      <c r="G8" s="37" t="inlineStr">
-        <is>
-          <t>customer_id, direction, amount, type</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>BRONZE</t>
-        </is>
-      </c>
-      <c r="C9" s="64" t="inlineStr">
-        <is>
-          <t>fact_card_transaction</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>~3,000,000</t>
-        </is>
-      </c>
-      <c r="E9" s="16" t="inlineStr">
-        <is>
-          <t>Fact</t>
-        </is>
-      </c>
-      <c r="F9" s="16" t="inlineStr">
-        <is>
-          <t>txn_id</t>
-        </is>
-      </c>
-      <c r="G9" s="36" t="inlineStr">
-        <is>
-          <t>amount, status, merchant, fraud_flag</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="21" t="inlineStr">
-        <is>
-          <t>BRONZE</t>
-        </is>
-      </c>
-      <c r="C10" s="65" t="inlineStr">
-        <is>
-          <t>fact_loan_application</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>200,000</t>
-        </is>
-      </c>
-      <c r="E10" s="19" t="inlineStr">
-        <is>
-          <t>Fact</t>
-        </is>
-      </c>
-      <c r="F10" s="19" t="inlineStr">
-        <is>
-          <t>loan_id</t>
-        </is>
-      </c>
-      <c r="G10" s="37" t="inlineStr">
-        <is>
-          <t>principal, decision, dpd, pd_score</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>BRONZE</t>
-        </is>
-      </c>
-      <c r="C11" s="64" t="inlineStr">
-        <is>
-          <t>fact_fx_rate</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>~95,000</t>
-        </is>
-      </c>
-      <c r="E11" s="16" t="inlineStr">
-        <is>
-          <t>Fact</t>
-        </is>
-      </c>
-      <c r="F11" s="16" t="inlineStr">
-        <is>
-          <t>rate_id</t>
-        </is>
-      </c>
-      <c r="G11" s="36" t="inlineStr">
-        <is>
-          <t>corridor, interbank, applied, spread_pct</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="21" t="inlineStr">
-        <is>
-          <t>BRONZE</t>
-        </is>
-      </c>
-      <c r="C12" s="65" t="inlineStr">
-        <is>
-          <t>fact_insurance_policy</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>40,000</t>
-        </is>
-      </c>
-      <c r="E12" s="19" t="inlineStr">
-        <is>
-          <t>Fact</t>
-        </is>
-      </c>
-      <c r="F12" s="19" t="inlineStr">
-        <is>
-          <t>policy_id</t>
-        </is>
-      </c>
-      <c r="G12" s="37" t="inlineStr">
-        <is>
-          <t>product, premium, status</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>BRONZE</t>
-        </is>
-      </c>
-      <c r="C13" s="64" t="inlineStr">
-        <is>
-          <t>fact_usd_savings</t>
-        </is>
-      </c>
-      <c r="D13" s="16" t="inlineStr">
-        <is>
-          <t>50,000</t>
-        </is>
-      </c>
-      <c r="E13" s="16" t="inlineStr">
-        <is>
-          <t>Fact</t>
-        </is>
-      </c>
-      <c r="F13" s="16" t="inlineStr">
-        <is>
-          <t>account_id</t>
-        </is>
-      </c>
-      <c r="G13" s="36" t="inlineStr">
-        <is>
-          <t>balance_zar, usdc_balance, status</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="25" t="inlineStr">
-        <is>
-          <t>SILVER</t>
-        </is>
-      </c>
-      <c r="C14" s="65" t="inlineStr">
-        <is>
-          <t>stg_transfers</t>
-        </is>
-      </c>
-      <c r="D14" s="19" t="inlineStr">
-        <is>
-          <t>view</t>
-        </is>
-      </c>
-      <c r="E14" s="19" t="inlineStr">
-        <is>
-          <t>dbt view</t>
-        </is>
-      </c>
-      <c r="F14" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G14" s="37" t="inlineStr">
-        <is>
-          <t>Cleaned transfers + derived fields</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="26" t="inlineStr">
-        <is>
-          <t>SILVER</t>
-        </is>
-      </c>
-      <c r="C15" s="64" t="inlineStr">
-        <is>
-          <t>int_transfer_profitability</t>
-        </is>
-      </c>
-      <c r="D15" s="16" t="inlineStr">
-        <is>
-          <t>~5M</t>
-        </is>
-      </c>
-      <c r="E15" s="16" t="inlineStr">
-        <is>
-          <t>dbt table</t>
-        </is>
-      </c>
-      <c r="F15" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G15" s="36" t="inlineStr">
-        <is>
-          <t>Transfers + FX join + margin tiers</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="25" t="inlineStr">
-        <is>
-          <t>SILVER</t>
-        </is>
-      </c>
-      <c r="C16" s="65" t="inlineStr">
-        <is>
-          <t>int_customer_transfer_stats</t>
-        </is>
-      </c>
-      <c r="D16" s="19" t="inlineStr">
-        <is>
-          <t>~500K</t>
-        </is>
-      </c>
-      <c r="E16" s="19" t="inlineStr">
-        <is>
-          <t>dbt table</t>
-        </is>
-      </c>
-      <c r="F16" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="37" t="inlineStr">
-        <is>
-          <t>Aggregated customer behaviour</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="B17" s="23" t="inlineStr">
-        <is>
-          <t>GOLD</t>
-        </is>
-      </c>
-      <c r="C17" s="64" t="inlineStr">
-        <is>
-          <t>mart_remittance</t>
-        </is>
-      </c>
-      <c r="D17" s="16" t="inlineStr">
-        <is>
-          <t>~50K</t>
-        </is>
-      </c>
-      <c r="E17" s="16" t="inlineStr">
-        <is>
-          <t>dbt table</t>
-        </is>
-      </c>
-      <c r="F17" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G17" s="36" t="inlineStr">
-        <is>
-          <t>Monthly corridor KPIs + revenue</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="24" t="inlineStr">
-        <is>
-          <t>GOLD</t>
-        </is>
-      </c>
-      <c r="C18" s="65" t="inlineStr">
-        <is>
-          <t>mart_customer_360</t>
-        </is>
-      </c>
-      <c r="D18" s="19" t="inlineStr">
-        <is>
-          <t>~500K</t>
-        </is>
-      </c>
-      <c r="E18" s="19" t="inlineStr">
-        <is>
-          <t>dbt table</t>
-        </is>
-      </c>
-      <c r="F18" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="37" t="inlineStr">
-        <is>
-          <t>One row per customer + LTV/engagement</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="B19" s="23" t="inlineStr">
-        <is>
-          <t>GOLD</t>
-        </is>
-      </c>
-      <c r="C19" s="64" t="inlineStr">
-        <is>
-          <t>mart_fx_profitability</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="inlineStr">
-        <is>
-          <t>~200</t>
-        </is>
-      </c>
-      <c r="E19" s="16" t="inlineStr">
-        <is>
-          <t>dbt table</t>
-        </is>
-      </c>
-      <c r="F19" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G19" s="36" t="inlineStr">
-        <is>
-          <t>Corridor FX margin by month</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="B20" s="24" t="inlineStr">
-        <is>
-          <t>GOLD</t>
-        </is>
-      </c>
-      <c r="C20" s="65" t="inlineStr">
-        <is>
-          <t>mart_risk_compliance</t>
-        </is>
-      </c>
-      <c r="D20" s="19" t="inlineStr">
-        <is>
-          <t>~12</t>
-        </is>
-      </c>
-      <c r="E20" s="19" t="inlineStr">
-        <is>
-          <t>dbt table</t>
-        </is>
-      </c>
-      <c r="F20" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G20" s="37" t="inlineStr">
-        <is>
-          <t>Monthly risk RAG status KPIs</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="23" t="inlineStr">
-        <is>
-          <t>GOLD</t>
-        </is>
-      </c>
-      <c r="C21" s="64" t="inlineStr">
-        <is>
-          <t>mart_loans_mukuru</t>
-        </is>
-      </c>
-      <c r="D21" s="16" t="inlineStr">
-        <is>
-          <t>~1K</t>
-        </is>
-      </c>
-      <c r="E21" s="16" t="inlineStr">
-        <is>
-          <t>dbt table</t>
-        </is>
-      </c>
-      <c r="F21" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G21" s="36" t="inlineStr">
-        <is>
-          <t>Loan origination + ECL + repayment</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="66" t="inlineStr">
-        <is>
-          <t>ML_DB</t>
-        </is>
-      </c>
-      <c r="C22" s="65" t="inlineStr">
-        <is>
-          <t>FRAUD_FEATURES</t>
-        </is>
-      </c>
-      <c r="D22" s="19" t="inlineStr">
-        <is>
-          <t>~200K</t>
-        </is>
-      </c>
-      <c r="E22" s="19" t="inlineStr">
-        <is>
-          <t>Feature table</t>
-        </is>
-      </c>
-      <c r="F22" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G22" s="37" t="inlineStr">
-        <is>
-          <t>15 fraud features refreshed daily</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="B23" s="67" t="inlineStr">
-        <is>
-          <t>ML_DB</t>
-        </is>
-      </c>
-      <c r="C23" s="64" t="inlineStr">
-        <is>
-          <t>CHURN_FEATURES</t>
-        </is>
-      </c>
-      <c r="D23" s="16" t="inlineStr">
-        <is>
-          <t>~500K</t>
-        </is>
-      </c>
-      <c r="E23" s="16" t="inlineStr">
-        <is>
-          <t>Feature table</t>
-        </is>
-      </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G23" s="36" t="inlineStr">
-        <is>
-          <t>21 churn features refreshed weekly</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B1:K2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>